<commit_message>
Review Anova and docs
</commit_message>
<xml_diff>
--- a/example/Config_link_windows_clean.xlsx
+++ b/example/Config_link_windows_clean.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -515,17 +515,17 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>C:/Users/forgi/OneDrive - Université de Namur/MASTER 2/Memoire/rnra_gui/example/20260430\250317</t>
+          <t>C:\Users\forgi\OneDrive - Université de Namur\MASTER 2\Memoire\rnra_gui\src\..\data\temp\250317</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>2.948312783327458</v>
+        <v>2.949101315820768</v>
       </c>
       <c r="J2" t="n">
-        <v>-8.088918884032058</v>
+        <v>-8.517423412978149</v>
       </c>
       <c r="K2" t="n">
-        <v>0.328839764380488</v>
+        <v>0.3267565101565981</v>
       </c>
     </row>
     <row r="3">
@@ -558,17 +558,17 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>C:/Users/forgi/OneDrive - Université de Namur/MASTER 2/Memoire/rnra_gui/example/20260430\250317</t>
+          <t>C:\Users\forgi\OneDrive - Université de Namur\MASTER 2\Memoire\rnra_gui\src\..\data\temp\250317</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>2.948312783327458</v>
+        <v>2.949101315820768</v>
       </c>
       <c r="J3" t="n">
-        <v>-8.088918884032058</v>
+        <v>-8.517423412978149</v>
       </c>
       <c r="K3" t="n">
-        <v>0.328839764380488</v>
+        <v>0.3267565101565981</v>
       </c>
     </row>
     <row r="4">
@@ -604,178 +604,6 @@
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>251112_1</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>C:\Users\forgi\OneDrive - Université de Namur\MASTER 2\Memoire\data\data\251112\251112\251112</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>C:\Users\forgi\OneDrive - Université de Namur\MASTER 2\Memoire\251112.xlsx.url</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" t="n">
-        <v>4</v>
-      </c>
-      <c r="F5" t="n">
-        <v>20</v>
-      </c>
-      <c r="G5" t="n">
-        <v>251112</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>C:/Users/forgi/OneDrive - Université de Namur/MASTER 2/Memoire/rnra_gui/example/20260430\251112</t>
-        </is>
-      </c>
-      <c r="I5" t="n">
-        <v>3.400911007294158</v>
-      </c>
-      <c r="J5" t="n">
-        <v>-11.72391201414656</v>
-      </c>
-      <c r="K5" t="n">
-        <v>0.382757438308858</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>251112_2</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>C:\Users\forgi\OneDrive - Université de Namur\MASTER 2\Memoire\data\data\251112\251112\251112</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>C:\Users\forgi\OneDrive - Université de Namur\MASTER 2\Memoire\251112.xlsx.url</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E6" t="n">
-        <v>21</v>
-      </c>
-      <c r="F6" t="n">
-        <v>32</v>
-      </c>
-      <c r="G6" t="n">
-        <v>251112</v>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>C:/Users/forgi/OneDrive - Université de Namur/MASTER 2/Memoire/rnra_gui/example/20260430\251112</t>
-        </is>
-      </c>
-      <c r="I6" t="n">
-        <v>3.400911007294158</v>
-      </c>
-      <c r="J6" t="n">
-        <v>-11.72391201414656</v>
-      </c>
-      <c r="K6" t="n">
-        <v>0.382757438308858</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>251112_3</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>C:\Users\forgi\OneDrive - Université de Namur\MASTER 2\Memoire\data\data\251112\251112\251112</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>C:\Users\forgi\OneDrive - Université de Namur\MASTER 2\Memoire\251112.xlsx.url</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E7" t="n">
-        <v>33</v>
-      </c>
-      <c r="F7" t="n">
-        <v>48</v>
-      </c>
-      <c r="G7" t="n">
-        <v>251112</v>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>C:/Users/forgi/OneDrive - Université de Namur/MASTER 2/Memoire/rnra_gui/example/20260430\251112</t>
-        </is>
-      </c>
-      <c r="I7" t="n">
-        <v>3.400911007294158</v>
-      </c>
-      <c r="J7" t="n">
-        <v>-11.72391201414656</v>
-      </c>
-      <c r="K7" t="n">
-        <v>0.382757438308858</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>251112_4</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>C:\Users\forgi\OneDrive - Université de Namur\MASTER 2\Memoire\data\data\251112\251112\251112</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>C:\Users\forgi\OneDrive - Université de Namur\MASTER 2\Memoire\251112.xlsx.url</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" t="n">
-        <v>49</v>
-      </c>
-      <c r="F8" t="n">
-        <v>61</v>
-      </c>
-      <c r="G8" t="n">
-        <v>251112</v>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>C:/Users/forgi/OneDrive - Université de Namur/MASTER 2/Memoire/rnra_gui/example/20260430\251112</t>
-        </is>
-      </c>
-      <c r="I8" t="n">
-        <v>3.400911007294158</v>
-      </c>
-      <c r="J8" t="n">
-        <v>-11.72391201414656</v>
-      </c>
-      <c r="K8" t="n">
-        <v>0.382757438308858</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>